<commit_message>
CCD-6251 Fix CaseTypeTab nested subfield fixture
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/CCD_BEFTA_CTT_LISTELEMENCODE.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/CCD_BEFTA_CTT_LISTELEMENCODE.xlsx
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2415" uniqueCount="521">
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2413" uniqueCount="521">
   <ns0:si>
     <ns0:t>UserProfile</ns0:t>
   </ns0:si>
@@ -2895,21 +2895,25 @@
       <c r="D15" t="s">
         <v>103</v>
       </c>
-      <c r="E15" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" t="s">
-        <v>107</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FamilyAddressDetails</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Family Address Details</t>
+        </is>
       </c>
       <c r="G15">
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Class.ClassDetails.ClassLocation.Building.Name</t>
+          <t>FamilyAddress.Country</t>
         </is>
       </c>
       <c r="J15">

</xml_diff>